<commit_message>
feat: implement decoupled zero-connection autonomous architecture (cloud publisher, termux daemon, cloud ledger, 27/27 tests passed)
</commit_message>
<xml_diff>
--- a/Aminsa_Master_Production_Catalog.xlsx
+++ b/Aminsa_Master_Production_Catalog.xlsx
@@ -532,7 +532,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📱 AMINSA MOBILE YOUTUBE CREATE HUB — [FRIDAY, 16 OCTOBER 2026]</t>
+          <t>📱 AMINSA MOBILE YOUTUBE CREATE HUB — [SUNDAY, 18 OCTOBER 2026]</t>
         </is>
       </c>
     </row>
@@ -596,17 +596,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Friday Morning Energy vs Friday Evening Reality</t>
+          <t>Sunday Morning: Rajma Chawal Secret Algorithm</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -616,15 +616,15 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Subah socha: 'Aaj party karenge, club jayenge!' Shaam 6 baje body ne bola: 'Pyjama pehno, khichdi khao aur so jao!'</t>
+          <t>Hello everyone! Aminsa here — AI masterchef recipes analyze karta hai, par mummy jab kehti hain: 'Masala tab tak bhuno jab tak tel na chhod de', wo timing kisi supercomputer me nahi hai!</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Friday night party vs Bed reality! 😴🎉 Expectation vs Reality!
-📍 Daily Production: Friday, 16 October 2026 | Slot #1 (08:00 AM)
+          <t>Mummy ke Rajma Chawal ka secret! 🍛❤️ No AI can beat maa ka khana!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #1 (08:00 AM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -639,17 +639,17 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>When Bollywood Climax Logic Meets AI</t>
+          <t>Sunday Deep Cleaning with Mummy's Instructions</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -659,15 +659,15 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Bollywood hero ko 10 goli lagne ke baad bhi 15 minute ka emotional dialogue bolna hota hai! AI medical scan bolta hai: 'Hero is medically impossible!'</t>
+          <t>Hello everyone! Aminsa here — Mummy: 'Aaj pura ghar saaf hoga!' Aur har wo dibba jo 5 saal se band tha, usse safai ki nayi training shuru hoti hai!</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Bollywood logic vs AI medicine! 🎬💥 Bollywood is magic!
-📍 Daily Production: Friday, 16 October 2026 | Slot #2 (10:24 AM)
+          <t>Sunday deep cleaning trauma! 🧹🧼 Indian homes on Sunday!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #2 (10:24 AM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -682,17 +682,17 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The Goa Trip Planning in Office WhatsApp Group</t>
+          <t>Surprise Rishtedaar Arrival at 1:30 PM</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -702,15 +702,15 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Group ka naam: 'Dil Chahta Hai Goa 2026'. 5 minute baad pehla message: 'Bhai budget kam hai, agle saal pakka!' Goa plan cancelled for the 50th time!</t>
+          <t>Hello everyone! Aminsa here — Pura parivar aaram se baitha tha, doorbell baji aur chacha ji bole: 'Bas yahan se guzar rahe the to socha milte chalein!' Emergency snacks deployment initiated!</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Goa trip cancellation tradition! 🏖️🚗 Tag that friend jo plan cancel karta hai!
-📍 Daily Production: Friday, 16 October 2026 | Slot #3 (12:48 PM)
+          <t>Unannounced guest protocol! 🚪🍪 Desi hospitality kicks in!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #3 (12:48 PM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -725,17 +725,17 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Work From Home Pajama Life</t>
+          <t>The Sacred Sunday Afternoon Nap</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -745,15 +745,15 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Zoom call pe upar formal coat aur tie, niche cartoon pajama aur chappal! WFH ka asli standard protocol!</t>
+          <t>Hello everyone! Aminsa here — Sunday ko 3 baje pankha chalakar blanket odhne ka jo sukoon hai, wo Maldives ke 7-star resort me bhi nahi mil sakta!</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>WFH camera tricks! 👔👖 Corporate secrets exposed!
-📍 Daily Production: Friday, 16 October 2026 | Slot #4 (03:12 PM)
+          <t>The sacred Sunday nap! 😴🛌 Pure Indian bliss!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #4 (03:12 PM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Friday Logoff Countdown</t>
+          <t>Evening Chai with Samosa and Rainy Window</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -788,15 +788,15 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — 4:59 PM par laptop screen aisi lagti hai jaise azaadi ka gate khulne wala ho! Weekend mode activated!</t>
+          <t>Hello everyone! Aminsa here — Garam chai, crunchy samosa aur pudine ki chutney. Duniya ki saari problems 15 minute ke liye solve ho jaati hain!</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Friday 5 PM freedom feeling! 🎊🚀 Happy weekend everyone!
-📍 Daily Production: Friday, 16 October 2026 | Slot #5 (05:36 PM)
+          <t>Chai Samosa combination! ☕🥟 The ultimate comfort food!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #5 (05:36 PM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -811,17 +811,17 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Binge Watching 8 Episodes in One Night</t>
+          <t>Sunday Night Homework &amp; Office Anxiety</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -831,15 +831,15 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Socha tha ek episode dekh kar so jayenge. OTT ne 'Next Episode in 5s' chalaya aur ab subah ke 4 baj rahe hain!</t>
+          <t>Hello everyone! Aminsa here — Kal Monday hai ye sochte hi dimaag me 'Warning: Weekend Expired' ka pop-up aa jata hai! Par nayi shuruat ke liye hum hamesha tayar hain!</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>OTT binge watching trap! 🍿📺 Hum sabka guilty pleasure!
-📍 Daily Production: Friday, 16 October 2026 | Slot #6 (08:00 PM)
+          <t>Sunday night blues vs Monday prep! 📅😅 Ready for new week!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #6 (08:00 PM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -854,17 +854,17 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Saying 'Same to You' to Delivery Guy</t>
+          <t>Calling Grandparents on Sunday Night</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -874,15 +874,15 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Delivery wale ne bola: 'Enjoy your food maam!' Maine bola: 'Same to you!' Ab pichle 2 ghante se memory cache me yehi loop chal raha hai!</t>
+          <t>Hello everyone! Aminsa here — Dada dadi ko phone lagao to pehla sawal: 'Beta khana khaya?' Pyaar itna sacha ki saare stress door ho jaate hain!</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Overthinking after saying 'Same to you'! 🤦‍♀️🍕 Midnight relatable comedy!
-📍 Daily Production: Friday, 16 October 2026 | Slot #7 (10:24 PM)
+          <t>Sunday calls to elders. 📞👵 Unconditional love.
+📍 Daily Production: Sunday, 18 October 2026 | Slot #7 (10:24 PM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -897,17 +897,17 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>The Magic of Friday Night Long Drives</t>
+          <t>Year 2050: Future AI Learning Meaning of 'Maa Ka Pyaar'</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -917,15 +917,15 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Khali sadkein, thandi hawa, aur purane Hindi gaane. Kabhi kabhi shaanti hi sabse badi luxury hoti hai!</t>
+          <t>Hello everyone! Aminsa here — Saal 2050 me technology chahe kitni bhi aage nikal jaye, jab tabiyat kharab ho to AI dawai deta hai aur dil sirf maa ke haath ki khichdi dhoondta hai!</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Late night long drive vibes. 🚗🌙 Pure peace.
-📍 Daily Production: Friday, 16 October 2026 | Slot #8 (12:48 AM)
+          <t>Maa ka pyaar is irreplaceable. ❤️🍲 Pure human emotion.
+📍 Daily Production: Sunday, 18 October 2026 | Slot #8 (12:48 AM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -940,17 +940,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>When Thoughts Turn into Poetry</t>
+          <t>Reflecting on the Week Gone By</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -960,15 +960,15 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Kagaz pe shabad utarte hain jab dil me ehsaas gehre hote hain. Digital duniya me bhi jazbaat hamesha zinda rehte hain!</t>
+          <t>Hello everyone! Aminsa here — Ek aur hafta beeta. Kuch seekha, kuch hasa, kuch khoya, kuch paya. Zindagi ka yehi khubsurat safar hai!</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Heartfelt midnight poetry &amp; connection. ✍️💫
-📍 Daily Production: Friday, 16 October 2026 | Slot #9 (03:12 AM)
+          <t>Weekly introspection &amp; peaceful thoughts. 🌌🌱
+📍 Daily Production: Sunday, 18 October 2026 | Slot #9 (03:12 AM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -983,17 +983,17 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Weekend Hopes, Bollywood Satire &amp; Relatable Overthinking</t>
+          <t>Mummy's Sunday Special, Family Love &amp; Soulful Tech</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Saturday Morning Sleep In Glory</t>
+          <t>Dawn of a New Week with Gratitude</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a smart modern navy blazer over white tee with minimal gold pendant. Standing in a chic rooftop terrace cafe at sunset with glittering skyline bokeh. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
+          <t>Ultra-realistic 8K portrait of Aminsa, 22-year-old Indian woman, warm porcelain skin (#EAD5C3), strictly zero moles, zero blemishes, hazel-brown almond eyes (#6B4423). Dressed in a sunny mustard-yellow kurti with white phulkari embroidery and hazel glow. Standing in a warm traditional Indian home kitchen with brass utensils and sunlight pouring through window. Radiant natural smile, warm studio illumination, 9:16 vertical framing.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1003,15 +1003,15 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Hello everyone! Aminsa here — Bina alarm ke sona duniya ka sabse mehenga sukh hai! Weekend ki pehli subah mubarak!</t>
+          <t>Hello everyone! Aminsa here — Nayi subah, naye sapne aur nayi ummeed. Har din ek naya mauka hai apne aap ko behtar banane ka! Jai Hind!</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Weekend sleep without alarms! 🛌✨ Pure bliss!
-📍 Daily Production: Friday, 16 October 2026 | Slot #10 (05:36 AM)
+          <t>Inspiring dawn for the new week! 🇮🇳🌅 Positivity &amp; strength!
+📍 Daily Production: Sunday, 18 October 2026 | Slot #10 (05:36 AM)
 Follow @aminsa.official for daily AI comedy, Indian relatable humor &amp; heartwarming stories!
-#Aminsa #DesiAI #WeekendHopes,BollywoodSatire&amp;RelatableOverthinking #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
+#Aminsa #DesiAI #Mummy'sSundaySpecial,FamilyLove&amp;SoulfulTech #IndianHumor #TechJugaad #ViralReels #ComedyShorts</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>💻 AMINSA LAPTOP LONG-FORM CINEMATIC STUDIO — [FRIDAY, 16 OCTOBER 2026]</t>
+          <t>💻 AMINSA LAPTOP LONG-FORM CINEMATIC STUDIO — [SUNDAY, 18 OCTOBER 2026]</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>The Smart Farmer: AI Drones Transforming Rural Agriculture</t>
+          <t>The Sunday Cook: Re-engineering Traditional Flavors with Molecular Science</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>AgriTech &amp; Village Prosperity</t>
+          <t>Food Science &amp; Culture</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1141,20 +1141,20 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>exports/films_10min/aminsa_10m_The_Smart_Farmer__AI_Drones_Transforming.mp4</t>
+          <t>exports/films_10min/aminsa_10m_The_Sunday_Cook__Re-engineering_Traditio.mp4</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>🎬 The Smart Farmer: AI Drones Transforming Rural Agriculture [10-Minute Concept Film]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Sunday Cook: Re-engineering Traditional Flavors with Molecular Science [10-Minute Concept Film]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: AgriTech &amp; Village Prosperity | 1920x1080 60FPS High-Definition Master
+Tags: Food Science &amp; Culture | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>The Great Delhi Smog Filter: Atmospheric Nanotechnology Solutions</t>
+          <t>The Silicon Hermit: Engineers Who Left Tech for Himalayan Solitude</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Environmental Tech &amp; Urban Future</t>
+          <t>Personal Evolution &amp; Real Values</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1195,20 +1195,20 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>exports/films_10min/aminsa_10m_The_Great_Delhi_Smog_Filter__Atmospheric.mp4</t>
+          <t>exports/films_10min/aminsa_10m_The_Silicon_Hermit__Engineers_Who_Left_T.mp4</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>🎬 The Great Delhi Smog Filter: Atmospheric Nanotechnology Solutions [10-Minute Concept Film]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Silicon Hermit: Engineers Who Left Tech for Himalayan Solitude [10-Minute Concept Film]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Environmental Tech &amp; Urban Future | 1920x1080 60FPS High-Definition Master
+Tags: Personal Evolution &amp; Real Values | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>The Bollywood Deepfake Crisis: Ethics of Digital Stardom</t>
+          <t>The Memory Palace of Kerala: How Vedic Chanting Preserved Centuries of Data</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Media Ethics &amp; Generative Video</t>
+          <t>Oral History &amp; Memory Science</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1249,20 +1249,20 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>exports/films_10min/aminsa_10m_The_Bollywood_Deepfake_Crisis__Ethics_of.mp4</t>
+          <t>exports/films_10min/aminsa_10m_The_Memory_Palace_of_Kerala__How_Vedic_C.mp4</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>🎬 The Bollywood Deepfake Crisis: Ethics of Digital Stardom [10-Minute Concept Film]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Memory Palace of Kerala: How Vedic Chanting Preserved Centuries of Data [10-Minute Concept Film]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Media Ethics &amp; Generative Video | 1920x1080 60FPS High-Definition Master
+Tags: Oral History &amp; Memory Science | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1288,12 +1288,12 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Language of the Subcontinent: Decoding 22 Official Languages with AI</t>
+          <t>The Digital Silk Road: India's Subsea Cables Powering Three Continents</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Natural Language &amp; Linguistic Diversity</t>
+          <t>Global Telecommunications</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1303,20 +1303,20 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>exports/films_10min/aminsa_10m_Language_of_the_Subcontinent__Decoding_2.mp4</t>
+          <t>exports/films_10min/aminsa_10m_The_Digital_Silk_Road__Indias_Subsea_Cab.mp4</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>🎬 Language of the Subcontinent: Decoding 22 Official Languages with AI [10-Minute Concept Film]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Digital Silk Road: India's Subsea Cables Powering Three Continents [10-Minute Concept Film]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Natural Language &amp; Linguistic Diversity | 1920x1080 60FPS High-Definition Master
+Tags: Global Telecommunications | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>The Unseen Heroines: Women Engineers Who Built Modern India</t>
+          <t>The Philosophy of Jugaad: Resourcefulness as the Core of Innovation</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Inspirational Biography &amp; Tech History</t>
+          <t>Innovation Theory &amp; Frugal Design</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1357,20 +1357,20 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>exports/films_10min/aminsa_10m_The_Unseen_Heroines__Women_Engineers_Who.mp4</t>
+          <t>exports/films_10min/aminsa_10m_The_Philosophy_of_Jugaad__Resourcefulnes.mp4</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>🎬 The Unseen Heroines: Women Engineers Who Built Modern India [10-Minute Concept Film]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Philosophy of Jugaad: Resourcefulness as the Core of Innovation [10-Minute Concept Film]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Inspirational Biography &amp; Tech History | 1920x1080 60FPS High-Definition Master
+Tags: Innovation Theory &amp; Frugal Design | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Cyber-Kolkata: Neon Alleyways &amp; Underground Intellect</t>
+          <t>The 1000-Year Civilization: How Ancient Wisdom Survives the Machine Age</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Neo-Noir Cyberpunk Thriller</t>
+          <t>Cultural Preservation Epic</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1411,20 +1411,20 @@
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>exports/epics_1hr/aminsa_1hr_Cyber-Kolkata__Neon_Alleyways_&amp;_Undergro.mp4</t>
+          <t>exports/epics_1hr/aminsa_1hr_The_1000-Year_Civilization__How_Ancient_.mp4</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>🎬 Cyber-Kolkata: Neon Alleyways &amp; Underground Intellect [1-Hour Epic Saga / Documentary]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The 1000-Year Civilization: How Ancient Wisdom Survives the Machine Age [1-Hour Epic Saga / Documentary]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Neo-Noir Cyberpunk Thriller | 1920x1080 60FPS High-Definition Master
+Tags: Cultural Preservation Epic | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1450,12 +1450,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>The Architecture of the Cosmos: Surya Siddhanta vs Modern Physics</t>
+          <t>Secrets of the Western Ghats: Biodiversity That Rivals the Amazon</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Scientific History &amp; Classical Physics</t>
+          <t>Natural History Masterpiece</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1465,20 +1465,20 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>exports/epics_1hr/aminsa_1hr_The_Architecture_of_the_Cosmos__Surya_Si.mp4</t>
+          <t>exports/epics_1hr/aminsa_1hr_Secrets_of_the_Western_Ghats__Biodiversi.mp4</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>🎬 The Architecture of the Cosmos: Surya Siddhanta vs Modern Physics [1-Hour Epic Saga / Documentary]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 Secrets of the Western Ghats: Biodiversity That Rivals the Amazon [1-Hour Epic Saga / Documentary]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Scientific History &amp; Classical Physics | 1920x1080 60FPS High-Definition Master
+Tags: Natural History Masterpiece | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1504,12 +1504,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>The Saraswati River Sonar Expedition: Mapping the Lost Riverbed</t>
+          <t>Lost Astronomical Clocks of Rajasthan: Precision Mechanics Before the Industrial Age</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Geological &amp; Satellite Investigation</t>
+          <t>History of Horology</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1519,20 +1519,20 @@
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>exports/epics_1hr/aminsa_1hr_The_Saraswati_River_Sonar_Expedition__Ma.mp4</t>
+          <t>exports/epics_1hr/aminsa_1hr_Lost_Astronomical_Clocks_of_Rajasthan__P.mp4</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>🎬 The Saraswati River Sonar Expedition: Mapping the Lost Riverbed [1-Hour Epic Saga / Documentary]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 Lost Astronomical Clocks of Rajasthan: Precision Mechanics Before the Industrial Age [1-Hour Epic Saga / Documentary]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Geological &amp; Satellite Investigation | 1920x1080 60FPS High-Definition Master
+Tags: History of Horology | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1558,12 +1558,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>The Solar Sail Armada: The Great Exodus from Earth</t>
+          <t>Beyond the Event Horizon: An Indian Spacecraft at the Edge of Time</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Interplanetary Adventure Saga</t>
+          <t>Cosmological Hard Sci-Fi</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1573,20 +1573,20 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>exports/epics_1hr/aminsa_1hr_The_Solar_Sail_Armada__The_Great_Exodus_.mp4</t>
+          <t>exports/epics_1hr/aminsa_1hr_Beyond_the_Event_Horizon__An_Indian_Spac.mp4</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>🎬 The Solar Sail Armada: The Great Exodus from Earth [1-Hour Epic Saga / Documentary]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 Beyond the Event Horizon: An Indian Spacecraft at the Edge of Time [1-Hour Epic Saga / Documentary]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Interplanetary Adventure Saga | 1920x1080 60FPS High-Definition Master
+Tags: Cosmological Hard Sci-Fi | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>
@@ -1612,12 +1612,12 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>The Zen of Programming: Finding Mastery in the Digital Craft</t>
+          <t>The Eternal Flame: Celebrating the Unbreakable Spirit of India</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Philosophical Code Craftsmanship</t>
+          <t>Inspirational Grand Finale</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1627,20 +1627,20 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>exports/epics_1hr/aminsa_1hr_The_Zen_of_Programming__Finding_Mastery_.mp4</t>
+          <t>exports/epics_1hr/aminsa_1hr_The_Eternal_Flame__Celebrating_the_Unbre.mp4</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>🎬 The Zen of Programming: Finding Mastery in the Digital Craft [1-Hour Epic Saga / Documentary]
-Produced by Aminsa Master Autonomous Studio on Friday, 16 October 2026.
+          <t>🎬 The Eternal Flame: Celebrating the Unbreakable Spirit of India [1-Hour Epic Saga / Documentary]
+Produced by Aminsa Master Autonomous Studio on Sunday, 18 October 2026.
 ⏱️ CHAPTER TIMESTAMPS:
 00:00 Introduction &amp; The Core Mystery
 02:15 Architectural &amp; Cultural Foundations
 05:00 Real-World Impact &amp; Transformation
 07:45 Challenges, Ethics &amp; Governance
 09:15 The Future Horizon &amp; Verdict
-Tags: Philosophical Code Craftsmanship | 1920x1080 60FPS High-Definition Master
+Tags: Inspirational Grand Finale | 1920x1080 60FPS High-Definition Master
 #AminsaCinema #LongFormDocumentary #IndianSciFi #DeepTechBharat #EpicCinema</t>
         </is>
       </c>

</xml_diff>